<commit_message>
feat: adapting for v2 of the training
</commit_message>
<xml_diff>
--- a/dist/reports/analysis-history-template.xlsx
+++ b/dist/reports/analysis-history-template.xlsx
@@ -40,12 +40,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:BZ1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="3" width="24" customWidth="1"/>
     <col min="4" max="4" width="32" customWidth="1"/>
-    <col min="5" max="13" width="18" customWidth="1"/>
+    <col min="5" max="78" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -114,6 +114,331 @@
           <t>latency_ms</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>plant_count</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>aruco_marker_count</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>dataset_version</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>training_map50_mask</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>training_precision_mask</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>training_recall_mask</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>processed_image_width_px</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>processed_image_height_px</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>original_image_width_px</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>original_image_height_px</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>scale_calibrated</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>scale_reason</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>scale_dictionary</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>scale_marker_size_mm</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>scale_markers_detected</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>scale_yolo_markers_detected</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>scale_marker_ids</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>scale_average_side_px</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>scale_median_side_px</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>scale_mm_per_pixel</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>scale_pixels_per_mm</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>plant_height_count</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>plant_height_source_unit</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>plant_height_calibrated</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>plant_height_average_percent</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>plant_height_max_percent</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>plant_height_average_px</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>plant_height_max_px</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>plant_height_real_unit</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>plant_height_average_mm</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>plant_height_max_mm</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>leaf_size_count</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>leaf_size_source_unit</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>leaf_size_calibrated</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>leaf_average_width_percent</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>leaf_average_height_percent</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>leaf_average_area_percent</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>leaf_average_width_px</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>leaf_average_height_px</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>leaf_average_area_px2</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>leaf_size_real_unit</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>leaf_average_width_mm</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>leaf_average_height_mm</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>leaf_average_area_mm2</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>fruit_size_count</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>fruit_size_source_unit</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>fruit_size_calibrated</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>fruit_average_width_percent</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr">
+        <is>
+          <t>fruit_average_height_percent</t>
+        </is>
+      </c>
+      <c r="BK1" t="inlineStr">
+        <is>
+          <t>fruit_average_area_percent</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>fruit_average_width_px</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>fruit_average_height_px</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>fruit_average_area_px2</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>fruit_size_real_unit</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>fruit_average_width_mm</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>fruit_average_height_mm</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>fruit_average_area_mm2</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>fruit_states_method</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
+        <is>
+          <t>fruit_state_green_count</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>fruit_state_ripening_count</t>
+        </is>
+      </c>
+      <c r="BV1" t="inlineStr">
+        <is>
+          <t>fruit_state_ripe_count</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr">
+        <is>
+          <t>fruit_state_undefined_count</t>
+        </is>
+      </c>
+      <c r="BX1" t="inlineStr">
+        <is>
+          <t>fruit_states_counts</t>
+        </is>
+      </c>
+      <c r="BY1" t="inlineStr">
+        <is>
+          <t>detection_measurements_json</t>
+        </is>
+      </c>
+      <c r="BZ1" t="inlineStr">
+        <is>
+          <t>measurements_json</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>